<commit_message>
Weekly portfolio data update (2026-09-14)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>31.39</v>
+        <v>31.53</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0395</v>
+        <v>0.0393</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>32.04</v>
+        <v>31.77</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0408</v>
+        <v>0.0412</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>40.49</v>
+        <v>41.99</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0404</v>
+        <v>0.0312</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>17.63</v>
+        <v>17.41</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1066</v>
+        <v>0.108</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>5.38</v>
+        <v>2.71</v>
       </c>
       <c r="I18" s="13">
         <f>E18+F18</f>
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1530,6 +1530,142 @@
         <v>52.89</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" t="n">
+        <v>31.53</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0393</v>
+      </c>
+      <c r="H18" t="n">
+        <v>189.18</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="n">
+        <v>31.77</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0.0412</v>
+      </c>
+      <c r="H19" t="n">
+        <v>158.87</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" t="n">
+        <v>41.99</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="H20" t="n">
+        <v>335.88</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>17.41</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="H21" t="n">
+        <v>52.23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly portfolio data update (2026-09-21)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>31.53</v>
+        <v>31.73</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0393</v>
+        <v>0.0391</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>31.77</v>
+        <v>32.08</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0412</v>
+        <v>0.0408</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>41.99</v>
+        <v>41.26</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0312</v>
+        <v>0.0319</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>17.41</v>
+        <v>17.33</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.108</v>
+        <v>0.1085</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>2.71</v>
+        <v>2.72</v>
       </c>
       <c r="I18" s="13">
         <f>E18+F18</f>
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1666,6 +1666,142 @@
         <v>52.23</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" t="n">
+        <v>31.73</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>0.0391</v>
+      </c>
+      <c r="H22" t="n">
+        <v>190.38</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" t="n">
+        <v>32.08</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0.0408</v>
+      </c>
+      <c r="H23" t="n">
+        <v>160.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" t="n">
+        <v>41.26</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>0.0319</v>
+      </c>
+      <c r="H24" t="n">
+        <v>330.08</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>17.33</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0.1085</v>
+      </c>
+      <c r="H25" t="n">
+        <v>51.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly portfolio data update (2026-09-28)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>31.73</v>
+        <v>32.22</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0391</v>
+        <v>0.0385</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>32.08</v>
+        <v>31.85</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0408</v>
+        <v>0.0411</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>41.26</v>
+        <v>42.82</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0319</v>
+        <v>0.031</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>17.33</v>
+        <v>16.97</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1085</v>
+        <v>0.1108</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>2.72</v>
+        <v>2.75</v>
       </c>
       <c r="I18" s="13">
         <f>E18+F18</f>
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1802,6 +1802,142 @@
         <v>51.99</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" t="n">
+        <v>32.22</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="H26" t="n">
+        <v>193.32</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>31.85</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>0.0411</v>
+      </c>
+      <c r="H27" t="n">
+        <v>159.25</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" t="n">
+        <v>42.82</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="H28" t="n">
+        <v>342.56</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" t="n">
+        <v>16.97</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>0.1108</v>
+      </c>
+      <c r="H29" t="n">
+        <v>50.91</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly portfolio data update (2026-10-05)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>32.22</v>
+        <v>31.74</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0385</v>
+        <v>0.0391</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>31.85</v>
+        <v>30.97</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0411</v>
+        <v>0.0422</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>42.82</v>
+        <v>42.99</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.031</v>
+        <v>0.0314</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>16.97</v>
+        <v>16.74</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1108</v>
+        <v>0.1123</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -814,7 +814,9 @@
       <c r="G16" s="3" t="n">
         <v>3.06</v>
       </c>
-      <c r="H16" s="3" t="n"/>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="I16" s="13">
         <f>E16+F16</f>
         <v/>
@@ -844,6 +846,9 @@
       <c r="G17" t="n">
         <v>2</v>
       </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
       <c r="I17" s="13">
         <f>E17+F17</f>
         <v/>
@@ -873,6 +878,9 @@
       <c r="G18" t="n">
         <v>2.75</v>
       </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
       <c r="I18" s="13">
         <f>E18+F18</f>
         <v/>
@@ -901,6 +909,9 @@
       </c>
       <c r="G19" t="n">
         <v>1.41</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
       </c>
       <c r="I19" s="13">
         <f>E19+F19</f>
@@ -931,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1938,6 +1949,142 @@
         <v>50.91</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" t="n">
+        <v>31.74</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>0.0391</v>
+      </c>
+      <c r="H30" t="n">
+        <v>190.44</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>30.97</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>0.0422</v>
+      </c>
+      <c r="H31" t="n">
+        <v>154.85</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>8</v>
+      </c>
+      <c r="E32" t="n">
+        <v>42.99</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>0.0314</v>
+      </c>
+      <c r="H32" t="n">
+        <v>343.88</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>0.1123</v>
+      </c>
+      <c r="H33" t="n">
+        <v>50.22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly portfolio data update (2026-10-12)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>31.74</v>
+        <v>31.63</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0391</v>
+        <v>0.0392</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>30.97</v>
+        <v>29.88</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0422</v>
+        <v>0.0438</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>42.99</v>
+        <v>45.52</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0314</v>
+        <v>0.0297</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>16.74</v>
+        <v>16.51</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1123</v>
+        <v>0.1139</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -942,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -2085,6 +2085,142 @@
         <v>50.22</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="n">
+        <v>31.63</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>0.0392</v>
+      </c>
+      <c r="H34" t="n">
+        <v>189.78</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>0.0438</v>
+      </c>
+      <c r="H35" t="n">
+        <v>149.38</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>8</v>
+      </c>
+      <c r="E36" t="n">
+        <v>45.52</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0.0297</v>
+      </c>
+      <c r="H36" t="n">
+        <v>364.16</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>16.51</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0.1139</v>
+      </c>
+      <c r="H37" t="n">
+        <v>49.53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>